<commit_message>
Add hours logged per ticket to FINRA report
Hours Logged column with section totals in the Excel, HTML and PDF
versions, plus total and per-assignee hours on the summary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XHMGcK5xcB3Aij8WoHrhN7
</commit_message>
<xml_diff>
--- a/reports/FINRA_Completed_Tickets.xlsx
+++ b/reports/FINRA_Completed_Tickets.xlsx
@@ -15,11 +15,11 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">'For Review'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'For Review'!$A$4:$G$7</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'For Review'!$A$4:$H$7</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'Other FINRA'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Other FINRA'!$A$4:$G$12</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Other FINRA'!$A$4:$H$12</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Prod Pod'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Prod Pod'!$A$4:$G$12</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Prod Pod'!$A$4:$H$12</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="109">
   <si>
     <t xml:space="preserve">FINRA — Completed Tickets Report</t>
   </si>
@@ -51,6 +51,9 @@
     <t xml:space="preserve">Prod Pod</t>
   </si>
   <si>
+    <t xml:space="preserve">Hours logged</t>
+  </si>
+  <si>
     <t xml:space="preserve">Status</t>
   </si>
   <si>
@@ -69,6 +72,9 @@
     <t xml:space="preserve">Team</t>
   </si>
   <si>
+    <t xml:space="preserve">Hours</t>
+  </si>
+  <si>
     <t xml:space="preserve">Shibi Ramaiyan</t>
   </si>
   <si>
@@ -120,6 +126,9 @@
     <t xml:space="preserve">• The ‘For Review’ tab lists 3 tickets not counted: 2 multi-client tickets that include FINRA, and 1 FINRA ticket that was reopened.</t>
   </si>
   <si>
+    <t xml:space="preserve">• Hours Logged is the total time logged on each ticket in Jira (all time, not only this period); subtasks: none on these tickets.</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Last Updated is the ticket's last-updated date in Jira. Totals are live formulas over the Prod Pod and Other FINRA tabs.</t>
   </si>
   <si>
@@ -141,6 +150,9 @@
     <t xml:space="preserve">Last Updated</t>
   </si>
   <si>
+    <t xml:space="preserve">Hours Logged</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
@@ -214,6 +226,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total hours logged</t>
   </si>
   <si>
     <t xml:space="preserve">Other FINRA Completed Tickets</t>
@@ -349,11 +364,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot; h&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot; h&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot; h&quot;;;&quot;0 h&quot;"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,6 +444,14 @@
       <b val="true"/>
       <sz val="22"/>
       <color rgb="FF0F766E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="22"/>
+      <color rgb="FF7C3AED"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -559,6 +585,13 @@
     </font>
     <font>
       <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF94A3B8"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF94A3B8"/>
       <name val="Arial"/>
@@ -708,7 +741,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -741,43 +774,47 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -785,30 +822,34 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -817,56 +858,76 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -877,19 +938,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="30" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -901,11 +966,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1077,7 +1146,7 @@
       <rgbColor rgb="FF166534"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF7C3AED"/>
       <rgbColor rgb="FF0F766E"/>
       <rgbColor rgb="FFDCE6F7"/>
       <rgbColor rgb="FF878787"/>
@@ -1371,11 +1440,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="9975722"/>
-        <c:axId val="61007678"/>
+        <c:axId val="52735460"/>
+        <c:axId val="21513078"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9975722"/>
+        <c:axId val="52735460"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1407,7 +1476,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61007678"/>
+        <c:crossAx val="21513078"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1415,7 +1484,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61007678"/>
+        <c:axId val="21513078"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1481,7 +1550,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9975722"/>
+        <c:crossAx val="52735460"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1761,7 +1830,7 @@
     <tabColor rgb="FF14213D"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -1769,6 +1838,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1782,6 +1852,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -1794,6 +1865,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -1807,6 +1879,9 @@
       </c>
       <c r="D4" s="3" t="s">
         <v>5</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1826,231 +1901,267 @@
         <f aca="false">COUNTA('Prod Pod'!$C$5:$C$12)</f>
         <v>8</v>
       </c>
+      <c r="F5" s="8" t="n">
+        <f aca="false">SUM('Prod Pod'!$G$5:$G$12)+SUM('Other FINRA'!$G$5:$G$12)</f>
+        <v>60.58</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="9" t="s">
+      <c r="A8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="D8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="G8" s="11" t="s">
         <v>11</v>
       </c>
+      <c r="H8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$C$5:$C$12,A9)</f>
         <v>5</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="13" t="n">
         <f aca="false">COUNTIF('Other FINRA'!$C$5:$C$12,A9)</f>
         <v>7</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <f aca="false">B9+C9</f>
         <v>12</v>
       </c>
-      <c r="F9" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="12" t="n">
+      <c r="F9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$E$5:$E$12,F9)+COUNTIF('Other FINRA'!$E$5:$E$12,F9)</f>
         <v>7</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="15" t="s">
         <v>5</v>
       </c>
+      <c r="I9" s="16" t="n">
+        <f aca="false">SUMIF('Prod Pod'!$E$5:$E$12,F9,'Prod Pod'!$G$5:$G$12)+SUMIF('Other FINRA'!$E$5:$E$12,F9,'Other FINRA'!$G$5:$G$12)</f>
+        <v>36</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="12" t="n">
+      <c r="A10" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$C$5:$C$12,A10)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <f aca="false">COUNTIF('Other FINRA'!$C$5:$C$12,A10)</f>
         <v>1</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <f aca="false">B10+C10</f>
         <v>1</v>
       </c>
-      <c r="F10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="12" t="n">
+      <c r="F10" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$E$5:$E$12,F10)+COUNTIF('Other FINRA'!$E$5:$E$12,F10)</f>
         <v>1</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="15" t="s">
         <v>5</v>
       </c>
+      <c r="I10" s="16" t="n">
+        <f aca="false">SUMIF('Prod Pod'!$E$5:$E$12,F10,'Prod Pod'!$G$5:$G$12)+SUMIF('Other FINRA'!$E$5:$E$12,F10,'Other FINRA'!$G$5:$G$12)</f>
+        <v>17</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="12" t="n">
+      <c r="A11" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$C$5:$C$12,A11)</f>
         <v>1</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <f aca="false">COUNTIF('Other FINRA'!$C$5:$C$12,A11)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">B11+C11</f>
         <v>1</v>
       </c>
-      <c r="F11" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="12" t="n">
+      <c r="F11" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$E$5:$E$12,F11)+COUNTIF('Other FINRA'!$E$5:$E$12,F11)</f>
         <v>2</v>
       </c>
-      <c r="H11" s="18" t="s">
-        <v>17</v>
+      <c r="H11" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <f aca="false">SUMIF('Prod Pod'!$E$5:$E$12,F11,'Prod Pod'!$G$5:$G$12)+SUMIF('Other FINRA'!$E$5:$E$12,F11,'Other FINRA'!$G$5:$G$12)</f>
+        <v>2.75</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="12" t="n">
+      <c r="A12" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$C$5:$C$12,A12)</f>
         <v>2</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <f aca="false">COUNTIF('Other FINRA'!$C$5:$C$12,A12)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">B12+C12</f>
         <v>2</v>
       </c>
-      <c r="F12" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="12" t="n">
+      <c r="F12" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$E$5:$E$12,F12)+COUNTIF('Other FINRA'!$E$5:$E$12,F12)</f>
         <v>1</v>
       </c>
-      <c r="H12" s="18" t="s">
-        <v>17</v>
+      <c r="H12" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="16" t="n">
+        <f aca="false">SUMIF('Prod Pod'!$E$5:$E$12,F12,'Prod Pod'!$G$5:$G$12)+SUMIF('Other FINRA'!$E$5:$E$12,F12,'Other FINRA'!$G$5:$G$12)</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="12" t="n">
+      <c r="A13" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$C$5:$C$12,A13)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <f aca="false">COUNTIF('Other FINRA'!$C$5:$C$12,A13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">B13+C13</f>
         <v>0</v>
       </c>
-      <c r="F13" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="12" t="n">
+      <c r="F13" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$E$5:$E$12,F13)+COUNTIF('Other FINRA'!$E$5:$E$12,F13)</f>
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="s">
-        <v>17</v>
+      <c r="H13" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <f aca="false">SUMIF('Prod Pod'!$E$5:$E$12,F13,'Prod Pod'!$G$5:$G$12)+SUMIF('Other FINRA'!$E$5:$E$12,F13,'Other FINRA'!$G$5:$G$12)</f>
+        <v>1.08</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" s="22" t="n">
+      <c r="A14" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="24" t="n">
         <f aca="false">SUM(B9:B13)</f>
         <v>8</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">SUM(C9:C13)</f>
         <v>8</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="24" t="n">
         <f aca="false">SUM(D9:D13)</f>
         <v>16</v>
       </c>
-      <c r="F14" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" s="12" t="n">
+      <c r="F14" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="13" t="n">
         <f aca="false">COUNTIF('Prod Pod'!$E$5:$E$12,"Unassigned")+COUNTIF('Other FINRA'!$E$5:$E$12,"Unassigned")</f>
         <v>2</v>
       </c>
-      <c r="H14" s="18" t="s">
-        <v>17</v>
+      <c r="H14" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="16" t="n">
+        <f aca="false">SUMIF('Prod Pod'!$E$5:$E$12,F14,'Prod Pod'!$G$5:$G$12)+SUMIF('Other FINRA'!$E$5:$E$12,F14,'Other FINRA'!$G$5:$G$12)</f>
+        <v>3</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
-        <v>23</v>
+      <c r="A32" s="25" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="24" t="s">
-        <v>24</v>
+      <c r="A33" s="26" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="24" t="s">
-        <v>25</v>
+      <c r="A34" s="26" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="24" t="s">
-        <v>26</v>
+      <c r="A35" s="26" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="24" t="s">
-        <v>27</v>
+      <c r="A36" s="26" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="24" t="s">
-        <v>28</v>
+      <c r="A37" s="26" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="24" t="s">
-        <v>29</v>
+      <c r="A38" s="26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="26" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2069,235 +2180,279 @@
     <tabColor rgb="FF0F766E"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
+      <c r="A1" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
+      <c r="A2" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="A4" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="B4" s="30" t="s">
         <v>36</v>
       </c>
+      <c r="C4" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="31" t="s">
+      <c r="A5" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="33" t="s">
+      <c r="D5" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="34" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="36" t="n">
+        <v>17</v>
+      </c>
+      <c r="H5" s="32"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="30"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="31" t="s">
+      <c r="F6" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="38"/>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="36" t="s">
+      <c r="D7" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" s="35"/>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="31" t="s">
+      <c r="E7" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="32"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="G7" s="30"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="31" t="s">
+      <c r="D8" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="38"/>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="35"/>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" s="30"/>
+      <c r="D9" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="32"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" s="41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H10" s="38"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="H11" s="32"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H12" s="38"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46" t="n">
+        <f aca="false">SUM(G5:G12)</f>
         <v>53</v>
       </c>
-      <c r="B10" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" s="35"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="39" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="G11" s="30"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="39" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="36" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" s="35"/>
+      <c r="H13" s="45"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G12"/>
+  <autoFilter ref="A4:H12"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A5" r:id="rId1" display="CR-1274"/>
@@ -2326,239 +2481,283 @@
     <tabColor rgb="FF2B59C3"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="40" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
+      <c r="A1" s="47" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
+      <c r="A2" s="48" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="A4" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="B4" s="30" t="s">
         <v>36</v>
       </c>
+      <c r="C4" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="31" t="s">
+      <c r="A5" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" s="36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H5" s="32"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="49" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="38"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="32"/>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="38"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9" s="36" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H9" s="32"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="41" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H10" s="38"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="36" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H11" s="51" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="49" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="53" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" s="30"/>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="G6" s="35"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7" s="30"/>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="36" t="s">
-        <v>74</v>
-      </c>
-      <c r="G8" s="35"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="G9" s="30"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="35" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="G10" s="35"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="G11" s="43" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="44" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="G12" s="45" t="s">
-        <v>87</v>
-      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46" t="n">
+        <f aca="false">SUM(G5:G12)</f>
+        <v>7.58</v>
+      </c>
+      <c r="H13" s="45"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G12"/>
+  <autoFilter ref="A4:H12"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A5" r:id="rId1" display="CBT-146"/>
@@ -2587,136 +2786,165 @@
     <tabColor rgb="FF64748B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="A1" s="54" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="47" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
+      <c r="A2" s="55" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="A4" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="B4" s="30" t="s">
         <v>36</v>
       </c>
+      <c r="C4" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="31" t="s">
+      <c r="A5" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="56" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="51" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6" s="41" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H6" s="53" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="G7" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="51" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="48" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="G5" s="43" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="36" t="s">
-        <v>96</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>97</v>
-      </c>
-      <c r="G6" s="45" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="G7" s="43" t="s">
-        <v>103</v>
-      </c>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="46" t="n">
+        <f aca="false">SUM(G5:G7)</f>
+        <v>4.17</v>
+      </c>
+      <c r="H8" s="45"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G7"/>
+  <autoFilter ref="A4:H7"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A5" r:id="rId1" display="CBT-138"/>

</xml_diff>